<commit_message>
UK daily ratings for 2026-05-11
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-11.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-11.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P258"/>
+  <dimension ref="A1:P318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6182,17 +6182,17 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Fast Tara (IRE)</t>
+          <t>Mercurial (IRE)</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J98" t="n">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="K98" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="n">
@@ -6236,17 +6236,17 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Mercurial (IRE)</t>
+          <t>Fast Tara (IRE)</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J99" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="K99" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="n">
@@ -14230,36 +14230,34 @@
         <v>4</v>
       </c>
       <c r="G236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>Wild Thoughts (IRE)</t>
+          <t>Cashbox (IRE)</t>
         </is>
       </c>
       <c r="I236" t="n">
         <v>3</v>
       </c>
       <c r="J236" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K236" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L236" t="inlineStr"/>
       <c r="M236" t="n">
         <v>102.04</v>
       </c>
-      <c r="N236" t="n">
-        <v>78.3</v>
-      </c>
+      <c r="N236" t="inlineStr"/>
       <c r="O236" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P236" t="n">
-        <v>0</v>
+        <v>-13</v>
       </c>
     </row>
     <row r="237">
@@ -14288,30 +14286,28 @@
         <v>4</v>
       </c>
       <c r="G237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>Brave Hunter</t>
+          <t>Wild Thoughts (IRE)</t>
         </is>
       </c>
       <c r="I237" t="n">
         <v>3</v>
       </c>
       <c r="J237" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K237" t="n">
-        <v>78</v>
-      </c>
-      <c r="L237" t="n">
-        <v>1.5</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="L237" t="inlineStr"/>
       <c r="M237" t="n">
         <v>102.04</v>
       </c>
       <c r="N237" t="n">
-        <v>75.90000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -14348,30 +14344,30 @@
         <v>4</v>
       </c>
       <c r="G238" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>Magical Merlot</t>
+          <t>Brave Hunter</t>
         </is>
       </c>
       <c r="I238" t="n">
         <v>3</v>
       </c>
       <c r="J238" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K238" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L238" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="M238" t="n">
         <v>102.04</v>
       </c>
       <c r="N238" t="n">
-        <v>75</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -14408,30 +14404,30 @@
         <v>4</v>
       </c>
       <c r="G239" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>Abundant (IRE)</t>
+          <t>Magical Merlot</t>
         </is>
       </c>
       <c r="I239" t="n">
         <v>3</v>
       </c>
       <c r="J239" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K239" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L239" t="n">
-        <v>2.05</v>
+        <v>1.55</v>
       </c>
       <c r="M239" t="n">
         <v>102.04</v>
       </c>
       <c r="N239" t="n">
-        <v>74.09999999999999</v>
+        <v>75</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -14468,30 +14464,30 @@
         <v>4</v>
       </c>
       <c r="G240" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>Dumuji</t>
+          <t>Abundant (IRE)</t>
         </is>
       </c>
       <c r="I240" t="n">
         <v>3</v>
       </c>
       <c r="J240" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K240" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L240" t="n">
-        <v>3.05</v>
+        <v>2.05</v>
       </c>
       <c r="M240" t="n">
         <v>102.04</v>
       </c>
       <c r="N240" t="n">
-        <v>72</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -14528,30 +14524,30 @@
         <v>4</v>
       </c>
       <c r="G241" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Akho Mezzna (FR)</t>
+          <t>Dumuji</t>
         </is>
       </c>
       <c r="I241" t="n">
         <v>3</v>
       </c>
       <c r="J241" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K241" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L241" t="n">
-        <v>6.05</v>
+        <v>3.05</v>
       </c>
       <c r="M241" t="n">
         <v>102.04</v>
       </c>
       <c r="N241" t="n">
-        <v>64.7</v>
+        <v>72</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -14588,30 +14584,30 @@
         <v>4</v>
       </c>
       <c r="G242" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>Berkshire Boom (IRE)</t>
+          <t>Akho Mezzna (FR)</t>
         </is>
       </c>
       <c r="I242" t="n">
         <v>3</v>
       </c>
       <c r="J242" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K242" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="L242" t="n">
-        <v>6.2</v>
+        <v>6.05</v>
       </c>
       <c r="M242" t="n">
         <v>102.04</v>
       </c>
       <c r="N242" t="n">
-        <v>61.4</v>
+        <v>64.7</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -14619,7 +14615,7 @@
         </is>
       </c>
       <c r="P242" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="243">
@@ -14648,30 +14644,30 @@
         <v>4</v>
       </c>
       <c r="G243" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Annastarzy</t>
+          <t>Berkshire Boom (IRE)</t>
         </is>
       </c>
       <c r="I243" t="n">
         <v>3</v>
       </c>
       <c r="J243" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K243" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L243" t="n">
-        <v>6.95</v>
+        <v>6.2</v>
       </c>
       <c r="M243" t="n">
         <v>102.04</v>
       </c>
       <c r="N243" t="n">
-        <v>61.8</v>
+        <v>61.4</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -14679,7 +14675,7 @@
         </is>
       </c>
       <c r="P243" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="244">
@@ -14708,30 +14704,30 @@
         <v>4</v>
       </c>
       <c r="G244" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>Ohara</t>
+          <t>Annastarzy</t>
         </is>
       </c>
       <c r="I244" t="n">
         <v>3</v>
       </c>
       <c r="J244" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K244" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L244" t="n">
-        <v>8.449999999999999</v>
+        <v>6.95</v>
       </c>
       <c r="M244" t="n">
         <v>102.04</v>
       </c>
       <c r="N244" t="n">
-        <v>59.5</v>
+        <v>61.8</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -14739,7 +14735,7 @@
         </is>
       </c>
       <c r="P244" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245">
@@ -14772,17 +14768,17 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Cashbox (IRE)</t>
+          <t>Ohara</t>
         </is>
       </c>
       <c r="I245" t="n">
         <v>3</v>
       </c>
       <c r="J245" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K245" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L245" t="n">
         <v>8.449999999999999</v>
@@ -14791,7 +14787,7 @@
         <v>102.04</v>
       </c>
       <c r="N245" t="n">
-        <v>60.3</v>
+        <v>59.5</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -14859,7 +14855,7 @@
         </is>
       </c>
       <c r="P246" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247">
@@ -14919,7 +14915,7 @@
         </is>
       </c>
       <c r="P247" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248">
@@ -14979,7 +14975,7 @@
         </is>
       </c>
       <c r="P248" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249">
@@ -15578,6 +15574,3582 @@
       </c>
       <c r="P258" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>1</v>
+      </c>
+      <c r="C259" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>5</v>
+      </c>
+      <c r="G259" t="n">
+        <v>0</v>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Taseem</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>2</v>
+      </c>
+      <c r="J259" t="n">
+        <v>130</v>
+      </c>
+      <c r="K259" t="n">
+        <v>0</v>
+      </c>
+      <c r="L259" t="inlineStr"/>
+      <c r="M259" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P259" t="n">
+        <v>-12.5</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>1</v>
+      </c>
+      <c r="C260" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>5</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Arcadian Days</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>2</v>
+      </c>
+      <c r="J260" t="n">
+        <v>125</v>
+      </c>
+      <c r="K260" t="n">
+        <v>0</v>
+      </c>
+      <c r="L260" t="inlineStr"/>
+      <c r="M260" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P260" t="n">
+        <v>-12.5</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>1</v>
+      </c>
+      <c r="C261" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>5</v>
+      </c>
+      <c r="G261" t="n">
+        <v>1</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Indian Land</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>2</v>
+      </c>
+      <c r="J261" t="n">
+        <v>130</v>
+      </c>
+      <c r="K261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L261" t="inlineStr"/>
+      <c r="M261" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N261" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P261" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>1</v>
+      </c>
+      <c r="C262" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>5</v>
+      </c>
+      <c r="G262" t="n">
+        <v>2</v>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Blakes Monarch (IRE)</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>2</v>
+      </c>
+      <c r="J262" t="n">
+        <v>133</v>
+      </c>
+      <c r="K262" t="n">
+        <v>0</v>
+      </c>
+      <c r="L262" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M262" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N262" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P262" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>1</v>
+      </c>
+      <c r="C263" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>5</v>
+      </c>
+      <c r="G263" t="n">
+        <v>3</v>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Cydney Sweenie</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>2</v>
+      </c>
+      <c r="J263" t="n">
+        <v>128</v>
+      </c>
+      <c r="K263" t="n">
+        <v>0</v>
+      </c>
+      <c r="L263" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M263" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N263" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P263" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>1</v>
+      </c>
+      <c r="C264" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>5</v>
+      </c>
+      <c r="G264" t="n">
+        <v>4</v>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Kach Above</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>2</v>
+      </c>
+      <c r="J264" t="n">
+        <v>130</v>
+      </c>
+      <c r="K264" t="n">
+        <v>0</v>
+      </c>
+      <c r="L264" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M264" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N264" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>1</v>
+      </c>
+      <c r="C265" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>5</v>
+      </c>
+      <c r="G265" t="n">
+        <v>5</v>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Parading</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>2</v>
+      </c>
+      <c r="J265" t="n">
+        <v>133</v>
+      </c>
+      <c r="K265" t="n">
+        <v>0</v>
+      </c>
+      <c r="L265" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="M265" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N265" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P265" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>1</v>
+      </c>
+      <c r="C266" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>5</v>
+      </c>
+      <c r="G266" t="n">
+        <v>6</v>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Dun Eideann</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>2</v>
+      </c>
+      <c r="J266" t="n">
+        <v>125</v>
+      </c>
+      <c r="K266" t="n">
+        <v>0</v>
+      </c>
+      <c r="L266" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M266" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N266" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P266" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>1</v>
+      </c>
+      <c r="C267" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>5</v>
+      </c>
+      <c r="G267" t="n">
+        <v>7</v>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Crystal Kraken</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>2</v>
+      </c>
+      <c r="J267" t="n">
+        <v>125</v>
+      </c>
+      <c r="K267" t="n">
+        <v>0</v>
+      </c>
+      <c r="L267" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="M267" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N267" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P267" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>1</v>
+      </c>
+      <c r="C268" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>5</v>
+      </c>
+      <c r="G268" t="n">
+        <v>8</v>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Agnes Hathaway</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>2</v>
+      </c>
+      <c r="J268" t="n">
+        <v>128</v>
+      </c>
+      <c r="K268" t="n">
+        <v>0</v>
+      </c>
+      <c r="L268" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="M268" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N268" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>1</v>
+      </c>
+      <c r="C269" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>5</v>
+      </c>
+      <c r="G269" t="n">
+        <v>9</v>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Allaboutthelunch</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>2</v>
+      </c>
+      <c r="J269" t="n">
+        <v>130</v>
+      </c>
+      <c r="K269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L269" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M269" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N269" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P269" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>1</v>
+      </c>
+      <c r="C270" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>5</v>
+      </c>
+      <c r="G270" t="n">
+        <v>10</v>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Emerald Bay (IRE)</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>2</v>
+      </c>
+      <c r="J270" t="n">
+        <v>133</v>
+      </c>
+      <c r="K270" t="n">
+        <v>0</v>
+      </c>
+      <c r="L270" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="M270" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N270" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P270" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>1</v>
+      </c>
+      <c r="C271" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>5</v>
+      </c>
+      <c r="G271" t="n">
+        <v>11</v>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Bad Baker</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>2</v>
+      </c>
+      <c r="J271" t="n">
+        <v>133</v>
+      </c>
+      <c r="K271" t="n">
+        <v>0</v>
+      </c>
+      <c r="L271" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="M271" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="N271" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P271" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>2</v>
+      </c>
+      <c r="C272" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>6</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Arch Legend</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>5</v>
+      </c>
+      <c r="J272" t="n">
+        <v>119</v>
+      </c>
+      <c r="K272" t="n">
+        <v>49</v>
+      </c>
+      <c r="L272" t="inlineStr"/>
+      <c r="M272" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P272" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>2</v>
+      </c>
+      <c r="C273" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>6</v>
+      </c>
+      <c r="G273" t="n">
+        <v>1</v>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Tuba</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>5</v>
+      </c>
+      <c r="J273" t="n">
+        <v>135</v>
+      </c>
+      <c r="K273" t="n">
+        <v>65</v>
+      </c>
+      <c r="L273" t="inlineStr"/>
+      <c r="M273" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N273" t="n">
+        <v>67</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P273" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>2</v>
+      </c>
+      <c r="C274" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>6</v>
+      </c>
+      <c r="G274" t="n">
+        <v>2</v>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Fine Print (IRE)</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>5</v>
+      </c>
+      <c r="J274" t="n">
+        <v>124</v>
+      </c>
+      <c r="K274" t="n">
+        <v>54</v>
+      </c>
+      <c r="L274" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M274" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N274" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P274" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>2</v>
+      </c>
+      <c r="C275" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>6</v>
+      </c>
+      <c r="G275" t="n">
+        <v>3</v>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>V Power</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>6</v>
+      </c>
+      <c r="J275" t="n">
+        <v>132</v>
+      </c>
+      <c r="K275" t="n">
+        <v>62</v>
+      </c>
+      <c r="L275" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="M275" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N275" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P275" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>2</v>
+      </c>
+      <c r="C276" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>6</v>
+      </c>
+      <c r="G276" t="n">
+        <v>4</v>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Green Team (FR)</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>7</v>
+      </c>
+      <c r="J276" t="n">
+        <v>132</v>
+      </c>
+      <c r="K276" t="n">
+        <v>62</v>
+      </c>
+      <c r="L276" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M276" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N276" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P276" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>2</v>
+      </c>
+      <c r="C277" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>6</v>
+      </c>
+      <c r="G277" t="n">
+        <v>5</v>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Lednikov</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>8</v>
+      </c>
+      <c r="J277" t="n">
+        <v>126</v>
+      </c>
+      <c r="K277" t="n">
+        <v>56</v>
+      </c>
+      <c r="L277" t="n">
+        <v>12.65</v>
+      </c>
+      <c r="M277" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N277" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P277" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>2</v>
+      </c>
+      <c r="C278" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>6</v>
+      </c>
+      <c r="G278" t="n">
+        <v>6</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Starshine Legend (IRE)</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>5</v>
+      </c>
+      <c r="J278" t="n">
+        <v>133</v>
+      </c>
+      <c r="K278" t="n">
+        <v>63</v>
+      </c>
+      <c r="L278" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="M278" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N278" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P278" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>2</v>
+      </c>
+      <c r="C279" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>6</v>
+      </c>
+      <c r="G279" t="n">
+        <v>7</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Sneaky Blinder (FR)</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>5</v>
+      </c>
+      <c r="J279" t="n">
+        <v>128</v>
+      </c>
+      <c r="K279" t="n">
+        <v>58</v>
+      </c>
+      <c r="L279" t="n">
+        <v>15.55</v>
+      </c>
+      <c r="M279" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N279" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P279" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>2</v>
+      </c>
+      <c r="C280" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>6</v>
+      </c>
+      <c r="G280" t="n">
+        <v>8</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Spec Of Light</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>4</v>
+      </c>
+      <c r="J280" t="n">
+        <v>130</v>
+      </c>
+      <c r="K280" t="n">
+        <v>60</v>
+      </c>
+      <c r="L280" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="M280" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N280" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P280" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>2</v>
+      </c>
+      <c r="C281" t="n">
+        <v>13.99545454545455</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>6</v>
+      </c>
+      <c r="G281" t="n">
+        <v>9</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Daaris (IRE)</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>7</v>
+      </c>
+      <c r="J281" t="n">
+        <v>132</v>
+      </c>
+      <c r="K281" t="n">
+        <v>62</v>
+      </c>
+      <c r="L281" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="M281" t="n">
+        <v>183.13</v>
+      </c>
+      <c r="N281" t="n">
+        <v>40</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P281" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>3</v>
+      </c>
+      <c r="C282" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>6</v>
+      </c>
+      <c r="G282" t="n">
+        <v>1</v>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Wave Rock (IRE)</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>4</v>
+      </c>
+      <c r="J282" t="n">
+        <v>135</v>
+      </c>
+      <c r="K282" t="n">
+        <v>59</v>
+      </c>
+      <c r="L282" t="inlineStr"/>
+      <c r="M282" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N282" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P282" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>3</v>
+      </c>
+      <c r="C283" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>6</v>
+      </c>
+      <c r="G283" t="n">
+        <v>2</v>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Merapi</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>4</v>
+      </c>
+      <c r="J283" t="n">
+        <v>135</v>
+      </c>
+      <c r="K283" t="n">
+        <v>59</v>
+      </c>
+      <c r="L283" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M283" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N283" t="n">
+        <v>47</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P283" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>3</v>
+      </c>
+      <c r="C284" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>6</v>
+      </c>
+      <c r="G284" t="n">
+        <v>3</v>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Arlecchinos Rex</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>4</v>
+      </c>
+      <c r="J284" t="n">
+        <v>127</v>
+      </c>
+      <c r="K284" t="n">
+        <v>51</v>
+      </c>
+      <c r="L284" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M284" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N284" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P284" t="n">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>3</v>
+      </c>
+      <c r="C285" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>6</v>
+      </c>
+      <c r="G285" t="n">
+        <v>4</v>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Book Of Life</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>6</v>
+      </c>
+      <c r="J285" t="n">
+        <v>133</v>
+      </c>
+      <c r="K285" t="n">
+        <v>57</v>
+      </c>
+      <c r="L285" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="M285" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N285" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P285" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>3</v>
+      </c>
+      <c r="C286" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>6</v>
+      </c>
+      <c r="G286" t="n">
+        <v>5</v>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Crafter (IRE)</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>8</v>
+      </c>
+      <c r="J286" t="n">
+        <v>131</v>
+      </c>
+      <c r="K286" t="n">
+        <v>55</v>
+      </c>
+      <c r="L286" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="M286" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N286" t="n">
+        <v>41</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P286" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>3</v>
+      </c>
+      <c r="C287" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>6</v>
+      </c>
+      <c r="G287" t="n">
+        <v>6</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Relevant Range (IRE)</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>7</v>
+      </c>
+      <c r="J287" t="n">
+        <v>135</v>
+      </c>
+      <c r="K287" t="n">
+        <v>59</v>
+      </c>
+      <c r="L287" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="M287" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N287" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P287" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>3</v>
+      </c>
+      <c r="C288" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>6</v>
+      </c>
+      <c r="G288" t="n">
+        <v>7</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Tiger Beetle</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>8</v>
+      </c>
+      <c r="J288" t="n">
+        <v>129</v>
+      </c>
+      <c r="K288" t="n">
+        <v>53</v>
+      </c>
+      <c r="L288" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M288" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N288" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P288" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>3</v>
+      </c>
+      <c r="C289" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>6</v>
+      </c>
+      <c r="G289" t="n">
+        <v>8</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Beat The Odds</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>4</v>
+      </c>
+      <c r="J289" t="n">
+        <v>121</v>
+      </c>
+      <c r="K289" t="n">
+        <v>45</v>
+      </c>
+      <c r="L289" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="M289" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N289" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P289" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>3</v>
+      </c>
+      <c r="C290" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>6</v>
+      </c>
+      <c r="G290" t="n">
+        <v>9</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Wicklow Way (IRE)</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>4</v>
+      </c>
+      <c r="J290" t="n">
+        <v>130</v>
+      </c>
+      <c r="K290" t="n">
+        <v>54</v>
+      </c>
+      <c r="L290" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="M290" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N290" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P290" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>3</v>
+      </c>
+      <c r="C291" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>6</v>
+      </c>
+      <c r="G291" t="n">
+        <v>10</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Molly Valentine (IRE)</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>6</v>
+      </c>
+      <c r="J291" t="n">
+        <v>134</v>
+      </c>
+      <c r="K291" t="n">
+        <v>58</v>
+      </c>
+      <c r="L291" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="M291" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N291" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P291" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>3</v>
+      </c>
+      <c r="C292" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>6</v>
+      </c>
+      <c r="G292" t="n">
+        <v>11</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Brinton</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>5</v>
+      </c>
+      <c r="J292" t="n">
+        <v>134</v>
+      </c>
+      <c r="K292" t="n">
+        <v>58</v>
+      </c>
+      <c r="L292" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="M292" t="n">
+        <v>122.62</v>
+      </c>
+      <c r="N292" t="n">
+        <v>27</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P292" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>4</v>
+      </c>
+      <c r="C293" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>3</v>
+      </c>
+      <c r="G293" t="n">
+        <v>1</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>She Commands (IRE)</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>3</v>
+      </c>
+      <c r="J293" t="n">
+        <v>135</v>
+      </c>
+      <c r="K293" t="n">
+        <v>0</v>
+      </c>
+      <c r="L293" t="inlineStr"/>
+      <c r="M293" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N293" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P293" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>4</v>
+      </c>
+      <c r="C294" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>3</v>
+      </c>
+      <c r="G294" t="n">
+        <v>2</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Wild Violet (FR)</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>3</v>
+      </c>
+      <c r="J294" t="n">
+        <v>128</v>
+      </c>
+      <c r="K294" t="n">
+        <v>0</v>
+      </c>
+      <c r="L294" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M294" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N294" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P294" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>4</v>
+      </c>
+      <c r="C295" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>3</v>
+      </c>
+      <c r="G295" t="n">
+        <v>3</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Celestra (FR)</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>3</v>
+      </c>
+      <c r="J295" t="n">
+        <v>128</v>
+      </c>
+      <c r="K295" t="n">
+        <v>81</v>
+      </c>
+      <c r="L295" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M295" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N295" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P295" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>4</v>
+      </c>
+      <c r="C296" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>3</v>
+      </c>
+      <c r="G296" t="n">
+        <v>4</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Hot Silk</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>3</v>
+      </c>
+      <c r="J296" t="n">
+        <v>128</v>
+      </c>
+      <c r="K296" t="n">
+        <v>0</v>
+      </c>
+      <c r="L296" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="M296" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N296" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P296" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>4</v>
+      </c>
+      <c r="C297" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>3</v>
+      </c>
+      <c r="G297" t="n">
+        <v>5</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Six Blue</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>6</v>
+      </c>
+      <c r="J297" t="n">
+        <v>142</v>
+      </c>
+      <c r="K297" t="n">
+        <v>0</v>
+      </c>
+      <c r="L297" t="n">
+        <v>8</v>
+      </c>
+      <c r="M297" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N297" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P297" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>4</v>
+      </c>
+      <c r="C298" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>3</v>
+      </c>
+      <c r="G298" t="n">
+        <v>6</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Musical Accord</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>3</v>
+      </c>
+      <c r="J298" t="n">
+        <v>128</v>
+      </c>
+      <c r="K298" t="n">
+        <v>0</v>
+      </c>
+      <c r="L298" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="M298" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="N298" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>5</v>
+      </c>
+      <c r="C299" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>6</v>
+      </c>
+      <c r="G299" t="n">
+        <v>1</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Street Dancer (IRE)</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>4</v>
+      </c>
+      <c r="J299" t="n">
+        <v>126</v>
+      </c>
+      <c r="K299" t="n">
+        <v>46</v>
+      </c>
+      <c r="L299" t="inlineStr"/>
+      <c r="M299" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N299" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P299" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>5</v>
+      </c>
+      <c r="C300" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>6</v>
+      </c>
+      <c r="G300" t="n">
+        <v>2</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>South Kensington (IRE)</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>5</v>
+      </c>
+      <c r="J300" t="n">
+        <v>135</v>
+      </c>
+      <c r="K300" t="n">
+        <v>55</v>
+      </c>
+      <c r="L300" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M300" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N300" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P300" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>5</v>
+      </c>
+      <c r="C301" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>6</v>
+      </c>
+      <c r="G301" t="n">
+        <v>3</v>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Captain Pickles (IRE)</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>4</v>
+      </c>
+      <c r="J301" t="n">
+        <v>135</v>
+      </c>
+      <c r="K301" t="n">
+        <v>55</v>
+      </c>
+      <c r="L301" t="n">
+        <v>7</v>
+      </c>
+      <c r="M301" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N301" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P301" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>5</v>
+      </c>
+      <c r="C302" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>6</v>
+      </c>
+      <c r="G302" t="n">
+        <v>4</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Shes A Goldigger</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>4</v>
+      </c>
+      <c r="J302" t="n">
+        <v>126</v>
+      </c>
+      <c r="K302" t="n">
+        <v>46</v>
+      </c>
+      <c r="L302" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="M302" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N302" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P302" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>5</v>
+      </c>
+      <c r="C303" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>6</v>
+      </c>
+      <c r="G303" t="n">
+        <v>5</v>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Simbas Gift</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>4</v>
+      </c>
+      <c r="J303" t="n">
+        <v>134</v>
+      </c>
+      <c r="K303" t="n">
+        <v>54</v>
+      </c>
+      <c r="L303" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="M303" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N303" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P303" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>5</v>
+      </c>
+      <c r="C304" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>6</v>
+      </c>
+      <c r="G304" t="n">
+        <v>6</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Princess Vivi</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>4</v>
+      </c>
+      <c r="J304" t="n">
+        <v>126</v>
+      </c>
+      <c r="K304" t="n">
+        <v>46</v>
+      </c>
+      <c r="L304" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="M304" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N304" t="n">
+        <v>58</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P304" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>5</v>
+      </c>
+      <c r="C305" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>6</v>
+      </c>
+      <c r="G305" t="n">
+        <v>7</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Love You More</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>4</v>
+      </c>
+      <c r="J305" t="n">
+        <v>134</v>
+      </c>
+      <c r="K305" t="n">
+        <v>54</v>
+      </c>
+      <c r="L305" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="M305" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N305" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P305" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>5</v>
+      </c>
+      <c r="C306" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>6</v>
+      </c>
+      <c r="G306" t="n">
+        <v>8</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Wyvern</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>7</v>
+      </c>
+      <c r="J306" t="n">
+        <v>132</v>
+      </c>
+      <c r="K306" t="n">
+        <v>52</v>
+      </c>
+      <c r="L306" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="M306" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N306" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P306" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>5</v>
+      </c>
+      <c r="C307" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>6</v>
+      </c>
+      <c r="G307" t="n">
+        <v>9</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Scarfo (IRE)</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>5</v>
+      </c>
+      <c r="J307" t="n">
+        <v>126</v>
+      </c>
+      <c r="K307" t="n">
+        <v>46</v>
+      </c>
+      <c r="L307" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="M307" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N307" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P307" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>5</v>
+      </c>
+      <c r="C308" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>6</v>
+      </c>
+      <c r="G308" t="n">
+        <v>10</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Aspire To Glory (IRE)</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>5</v>
+      </c>
+      <c r="J308" t="n">
+        <v>135</v>
+      </c>
+      <c r="K308" t="n">
+        <v>55</v>
+      </c>
+      <c r="L308" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="M308" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N308" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>5</v>
+      </c>
+      <c r="C309" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>6</v>
+      </c>
+      <c r="G309" t="n">
+        <v>11</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>So Chic (IRE)</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>6</v>
+      </c>
+      <c r="J309" t="n">
+        <v>131</v>
+      </c>
+      <c r="K309" t="n">
+        <v>51</v>
+      </c>
+      <c r="L309" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="M309" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N309" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P309" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>5</v>
+      </c>
+      <c r="C310" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>6</v>
+      </c>
+      <c r="G310" t="n">
+        <v>12</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Port Louis (IRE)</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>5</v>
+      </c>
+      <c r="J310" t="n">
+        <v>129</v>
+      </c>
+      <c r="K310" t="n">
+        <v>49</v>
+      </c>
+      <c r="L310" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="M310" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N310" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P310" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>5</v>
+      </c>
+      <c r="C311" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>6</v>
+      </c>
+      <c r="G311" t="n">
+        <v>13</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Red Admiral (IRE)</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>4</v>
+      </c>
+      <c r="J311" t="n">
+        <v>130</v>
+      </c>
+      <c r="K311" t="n">
+        <v>50</v>
+      </c>
+      <c r="L311" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="M311" t="n">
+        <v>107.39</v>
+      </c>
+      <c r="N311" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P311" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>6</v>
+      </c>
+      <c r="C312" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>5</v>
+      </c>
+      <c r="G312" t="n">
+        <v>1</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Crystal Pier (IRE)</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>3</v>
+      </c>
+      <c r="J312" t="n">
+        <v>133</v>
+      </c>
+      <c r="K312" t="n">
+        <v>73</v>
+      </c>
+      <c r="L312" t="inlineStr"/>
+      <c r="M312" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N312" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P312" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>6</v>
+      </c>
+      <c r="C313" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>5</v>
+      </c>
+      <c r="G313" t="n">
+        <v>2</v>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Lady Milton</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>3</v>
+      </c>
+      <c r="J313" t="n">
+        <v>131</v>
+      </c>
+      <c r="K313" t="n">
+        <v>71</v>
+      </c>
+      <c r="L313" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M313" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N313" t="n">
+        <v>72</v>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P313" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>6</v>
+      </c>
+      <c r="C314" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>5</v>
+      </c>
+      <c r="G314" t="n">
+        <v>3</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Silky Lass</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>3</v>
+      </c>
+      <c r="J314" t="n">
+        <v>128</v>
+      </c>
+      <c r="K314" t="n">
+        <v>68</v>
+      </c>
+      <c r="L314" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M314" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N314" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P314" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>6</v>
+      </c>
+      <c r="C315" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>5</v>
+      </c>
+      <c r="G315" t="n">
+        <v>4</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Squiffy (IRE)</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>4</v>
+      </c>
+      <c r="J315" t="n">
+        <v>136</v>
+      </c>
+      <c r="K315" t="n">
+        <v>62</v>
+      </c>
+      <c r="L315" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="M315" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N315" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P315" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>6</v>
+      </c>
+      <c r="C316" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>5</v>
+      </c>
+      <c r="G316" t="n">
+        <v>5</v>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Eastern Veil</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>3</v>
+      </c>
+      <c r="J316" t="n">
+        <v>135</v>
+      </c>
+      <c r="K316" t="n">
+        <v>75</v>
+      </c>
+      <c r="L316" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="M316" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N316" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P316" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>6</v>
+      </c>
+      <c r="C317" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>5</v>
+      </c>
+      <c r="G317" t="n">
+        <v>6</v>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Kilkenny Warrior (IRE)</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>3</v>
+      </c>
+      <c r="J317" t="n">
+        <v>135</v>
+      </c>
+      <c r="K317" t="n">
+        <v>75</v>
+      </c>
+      <c r="L317" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="M317" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N317" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P317" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>6</v>
+      </c>
+      <c r="C318" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>5</v>
+      </c>
+      <c r="G318" t="n">
+        <v>7</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Searchingtheblues</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>4</v>
+      </c>
+      <c r="J318" t="n">
+        <v>139</v>
+      </c>
+      <c r="K318" t="n">
+        <v>65</v>
+      </c>
+      <c r="L318" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M318" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="N318" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P318" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>